<commit_message>
Add sidenav metadata to Programs page and template importers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-programs-template.report.xlsx
+++ b/tools/importer/reports/import-programs-template.report.xlsx
@@ -97,7 +97,7 @@
     <t>programs</t>
   </si>
   <si>
-    <t>2026-10-29T00:32:12.147Z</t>
+    <t>2026-10-29T00:49:24.817Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/beedie/programs/undergraduate/bba-major/program.html</t>
@@ -124,7 +124,7 @@
     <t>landing-page</t>
   </si>
   <si>
-    <t>2026-10-28T07:31:46.139Z</t>
+    <t>2026-10-29T00:32:30.001Z</t>
   </si>
   <si>
     <t>templates/programs.report.json</t>
@@ -136,7 +136,7 @@
     <t>programs-template</t>
   </si>
   <si>
-    <t>2026-10-29T00:32:20.722Z</t>
+    <t>2026-10-29T00:49:33.239Z</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Rely on template defaults for sidenav: drop sidenav metadata from page importers
Programs and Resources templates already supply their navigation; pages only
need a sidenav metadata row to override it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-programs-template.report.xlsx
+++ b/tools/importer/reports/import-programs-template.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="55">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-29T00:30:29.725Z</t>
+    <t>2026-10-29T00:58:57.058Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -97,7 +97,7 @@
     <t>programs</t>
   </si>
   <si>
-    <t>2026-10-29T00:49:24.817Z</t>
+    <t>2026-10-29T01:19:49.954Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/beedie/programs/undergraduate/bba-major/program.html</t>
@@ -115,6 +115,33 @@
     <t>2026-10-29T00:31:18.120Z</t>
   </si>
   <si>
+    <t>fragments/resources-sidenav.report.json</t>
+  </si>
+  <si>
+    <t>fragments/resources-sidenav</t>
+  </si>
+  <si>
+    <t>resources-sidenav</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:58:29.131Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/research/researcher-resources/resources/research-facilities.html</t>
+  </si>
+  <si>
+    <t>resources/research-facilities.report.json</t>
+  </si>
+  <si>
+    <t>resources/research-facilities</t>
+  </si>
+  <si>
+    <t>resources</t>
+  </si>
+  <si>
+    <t>2026-10-29T01:00:14.429Z</t>
+  </si>
+  <si>
     <t>templates/landing-page.report.json</t>
   </si>
   <si>
@@ -136,7 +163,19 @@
     <t>programs-template</t>
   </si>
   <si>
-    <t>2026-10-29T00:49:33.239Z</t>
+    <t>2026-10-29T01:19:59.428Z</t>
+  </si>
+  <si>
+    <t>templates/resources.report.json</t>
+  </si>
+  <si>
+    <t>templates/resources</t>
+  </si>
+  <si>
+    <t>resources-template</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:58:47.210Z</t>
   </si>
 </sst>
 </file>
@@ -525,13 +564,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="1" max="1" width="43" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
     <col min="9" max="9" width="50" customWidth="1"/>
@@ -571,7 +610,7 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
@@ -766,36 +805,123 @@
         <v>11</v>
       </c>
       <c r="I8" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="s">
         <v>38</v>
       </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H9" t="s">
-        <v>11</v>
-      </c>
-      <c r="I9" t="s">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>